<commit_message>
actions worflow added and modified updated config file
</commit_message>
<xml_diff>
--- a/src/testdata/testdataReg.xlsx
+++ b/src/testdata/testdataReg.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\Opencart_WebFramework_PW\src\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A299A763-4374-4D3D-8189-21C7F3A146EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2697A2A4-3090-4B4F-9BB0-8193FD22C3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5F6219F4-288F-480C-8A60-B851487667E6}"/>
   </bookViews>
@@ -28,9 +28,6 @@
     <t>Kumar</t>
   </si>
   <si>
-    <t>naveen.kumar@testmail.com</t>
-  </si>
-  <si>
     <t>Test@1234</t>
   </si>
   <si>
@@ -43,9 +40,6 @@
     <t>Sharma</t>
   </si>
   <si>
-    <t>priya.sharma@testmail.com</t>
-  </si>
-  <si>
     <t>Pass123!</t>
   </si>
   <si>
@@ -58,9 +52,6 @@
     <t>Singh</t>
   </si>
   <si>
-    <t>rahul.singh@testmail.com</t>
-  </si>
-  <si>
     <t>Secure@22</t>
   </si>
   <si>
@@ -70,9 +61,6 @@
     <t>Rao</t>
   </si>
   <si>
-    <t>meena.rao@testmail.com</t>
-  </si>
-  <si>
     <t>Strong@55</t>
   </si>
   <si>
@@ -82,9 +70,6 @@
     <t>Doe</t>
   </si>
   <si>
-    <t>john.doe@testmail.com</t>
-  </si>
-  <si>
     <t>Abc@1234</t>
   </si>
   <si>
@@ -94,9 +79,6 @@
     <t>Patel</t>
   </si>
   <si>
-    <t>ananya.patel@testmail.com</t>
-  </si>
-  <si>
     <t>Welcome@9</t>
   </si>
   <si>
@@ -106,9 +88,6 @@
     <t>Reddy</t>
   </si>
   <si>
-    <t>vikram.reddy@testmail.com</t>
-  </si>
-  <si>
     <t>Hello@123</t>
   </si>
   <si>
@@ -118,9 +97,6 @@
     <t>Devi</t>
   </si>
   <si>
-    <t>sita.devi@testmail.com</t>
-  </si>
-  <si>
     <t>Pass@789</t>
   </si>
   <si>
@@ -130,9 +106,6 @@
     <t>Mehta</t>
   </si>
   <si>
-    <t>arjun.mehta@testmail.com</t>
-  </si>
-  <si>
     <t>Test@5678</t>
   </si>
   <si>
@@ -142,9 +115,6 @@
     <t>Nair</t>
   </si>
   <si>
-    <t>kiran.nair@testmail.com</t>
-  </si>
-  <si>
     <t>Valid@321</t>
   </si>
   <si>
@@ -197,13 +167,43 @@
   </si>
   <si>
     <t>1111111111</t>
+  </si>
+  <si>
+    <t>naveen.23qekumar@testmail.com</t>
+  </si>
+  <si>
+    <t>priya.sha23ewrma@testmail.com</t>
+  </si>
+  <si>
+    <t>rahul.si23dssangh@testmail.com</t>
+  </si>
+  <si>
+    <t>meena234ads.rao@testmail.com</t>
+  </si>
+  <si>
+    <t>john.dhs23oe@testmail.com</t>
+  </si>
+  <si>
+    <t>ananya.psdrrtatel@testmail.com</t>
+  </si>
+  <si>
+    <t>vikram.rewrweeddy@testmail.com</t>
+  </si>
+  <si>
+    <t>sita.desadfdsvi@testmail.com</t>
+  </si>
+  <si>
+    <t>arjun.mcvfehta@testmail.com</t>
+  </si>
+  <si>
+    <t>kiran.ndsfair@testmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,6 +334,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -636,7 +644,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
@@ -679,12 +687,14 @@
     <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
   </cellXfs>
-  <cellStyles count="42">
+  <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
     <cellStyle name="20% - Accent2" xfId="23" builtinId="34" customBuiltin="1"/>
     <cellStyle name="20% - Accent3" xfId="27" builtinId="38" customBuiltin="1"/>
@@ -718,6 +728,7 @@
     <cellStyle name="Heading 2" xfId="3" builtinId="17" customBuiltin="1"/>
     <cellStyle name="Heading 3" xfId="4" builtinId="18" customBuiltin="1"/>
     <cellStyle name="Heading 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Hyperlink" xfId="42" builtinId="8"/>
     <cellStyle name="Input" xfId="9" builtinId="20" customBuiltin="1"/>
     <cellStyle name="Linked Cell" xfId="12" builtinId="24" customBuiltin="1"/>
     <cellStyle name="Neutral" xfId="8" builtinId="28" customBuiltin="1"/>
@@ -1051,25 +1062,25 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="C1" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="E1" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="F1" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G1" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -1079,230 +1090,242 @@
       <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" t="s">
         <v>3</v>
-      </c>
-      <c r="F2" t="s">
-        <v>3</v>
-      </c>
-      <c r="G2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s">
+      <c r="F3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" t="s">
         <v>7</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" t="s">
         <v>10</v>
       </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
+        <v>12</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>52</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" t="s">
-        <v>20</v>
+        <v>15</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" t="s">
-        <v>24</v>
+        <v>18</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>54</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E7" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" t="s">
-        <v>28</v>
+        <v>21</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>55</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="F8" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="G8" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
+        <v>24</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>56</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
+        <v>27</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>57</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="E10" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="F10" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="G10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
+        <v>30</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>58</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="E11" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="F11" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="G11" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C2" r:id="rId1" xr:uid="{D69CEF91-BC90-4FE3-9678-539A286DB5D2}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{847E55A9-0CF0-4A80-BBA2-E4C09E5E1178}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{933A725F-8244-4949-AEFD-9F30EA8207E7}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{CBF70352-EE98-4DA9-A0CE-AE26E1908711}"/>
+    <hyperlink ref="C6" r:id="rId5" xr:uid="{520CE232-80E5-4749-83CA-3F7FAA209CC0}"/>
+    <hyperlink ref="C7" r:id="rId6" xr:uid="{6709F713-22DF-4C1C-8BCD-3843C375AD08}"/>
+    <hyperlink ref="C8" r:id="rId7" xr:uid="{A7EB3DD6-5977-439F-B8B6-2BA907FD92F5}"/>
+    <hyperlink ref="C9" r:id="rId8" xr:uid="{A487B4DB-2BE7-4FAF-A005-54D33047319D}"/>
+    <hyperlink ref="C10" r:id="rId9" xr:uid="{0A6F56C3-451F-4EE4-95B6-7B5BCE17060C}"/>
+    <hyperlink ref="C11" r:id="rId10" xr:uid="{5CA4E7CC-5538-452D-B8CC-3FE7D740F4DA}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>